<commit_message>
MultiFX's boot mode and the Alchemy Lab's panel, from their sources
The xlsx said MultiFX boots from QSPI with the Seed's low-pass in its
output; its Makefile says BOOT_NONE and its README says that filter is off
on the Patch SM. The Alchemy Lab's blank audio and control cells are filled
from the maker's page. MODULES.md notes the MultiFX unit is repurposed for
the neural-model experiment.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DM1Cn6bUpTT9LT2gqp5Yv9
</commit_message>
<xml_diff>
--- a/MCU_MODULES.xlsx
+++ b/MCU_MODULES.xlsx
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>128 KB internal + 8 MB QSPI (BOOT_QSPI)</t>
+          <t>128 KB internal + 8 MB QSPI (runs BOOT_NONE — internal flash, no bootloader)</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>Stereo L/R, with output voicing: DC-block → ~14.5 kHz LPF → soft clamp</t>
+          <t>Stereo L/R, with output voicing: DC-block → soft clamp (the Seed build's ~14.5 kHz LPF is disabled on the Patch SM)</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="U14" s="7" t="inlineStr">
         <is>
-          <t>daisy_multifx_oled/README.md</t>
+          <t>daisy_multifx_oled/README.md; daisy_multifx_oled/Makefile (APP_TYPE)</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Electrosmith Daisy — STM32H750</t>
+          <t>Electrosmith Daisy Seed 2 DFM — STM32H750</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -3220,7 +3220,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Internal + QSPI flash; MIT-licensed SDK</t>
+          <t>16 MB flash (per maker); MIT-licensed SDK (hermetic-modular/alchemy-sdk)</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
@@ -3235,12 +3235,12 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>USB</t>
+          <t>USB-C (MIDI)</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>USB-C MIDI</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
@@ -3255,22 +3255,22 @@
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
-          <t>Not recorded in the repos</t>
+          <t>Stereo L/R, up to 96 kHz / 24-bit</t>
         </is>
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
-          <t>Not recorded in the repos</t>
+          <t>Stereo L/R, up to 96 kHz / 24-bit</t>
         </is>
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>102 addressable LEDs</t>
+          <t>No screen — 102 addressable RGB LEDs</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>Not recorded in the repos</t>
+          <t>6 pots, 3 buttons; rear SPI / I2C expansion header</t>
         </is>
       </c>
       <c r="S30" s="7" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="U30" s="7" t="inlineStr">
         <is>
-          <t>MODULES.md</t>
+          <t>MODULES.md; hermeticmodular.com/modules/alchemy-lab and the Synth Anatomy launch article (2026-07), checked 2026-09-24</t>
         </is>
       </c>
     </row>

</xml_diff>